<commit_message>
Trim leading whitespace from imported anchor hrefs
Some source anchors carried a stray leading space in the href (e.g.
href=" https://www.addc.ae/..."). Left as-is the space became %20, and
the DA publish step then rewrote the whole value into a broken internal
path (/https/www-addc-ae/...), producing 404s on the overview pages.

Add an afterTransform rule to taqa-cleanup that trims surrounding
whitespace on every anchor href, and rebuild the residential import
bundle. Re-imported and re-published the 3 affected overview pages
(en-us/business, en-us/residential, ar-ae/business); all 15 links now
resolve as clean absolute addc.ae URLs.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-residential.report.xlsx
+++ b/tools/importer/reports/import-residential.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="115">
   <si>
     <t>_reportFile</t>
   </si>
@@ -121,7 +121,7 @@
     <t>residential</t>
   </si>
   <si>
-    <t>2026-09-22T06:52:36.690Z</t>
+    <t>2026-09-22T10:29:45.192Z</t>
   </si>
   <si>
     <t>TAQA Distribution</t>
@@ -136,7 +136,7 @@
     <t>addc/en-us/business/overview</t>
   </si>
   <si>
-    <t>2026-09-22T06:29:01.841Z</t>
+    <t>2026-09-22T10:29:29.986Z</t>
   </si>
   <si>
     <t>https://taqadistribution.com/addc/en-us/business/overview</t>
@@ -148,7 +148,7 @@
     <t>addc/en-us/residential/overview</t>
   </si>
   <si>
-    <t>2026-09-17T06:08:10.043Z</t>
+    <t>2026-09-22T10:29:38.734Z</t>
   </si>
   <si>
     <t>https://taqadistribution.com/addc/en-us/residential/overview</t>
@@ -220,6 +220,36 @@
     <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/transfer-and-removal-of-electricity-services</t>
   </si>
   <si>
+    <t>addc/ar-ae/business/locations/branches.report.json</t>
+  </si>
+  <si>
+    <t>["hero-text","cards-support"]</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/locations/branches</t>
+  </si>
+  <si>
+    <t>locations</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:53:02.465Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/locations/branches</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/locations/partners.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/locations/partners</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:53:12.213Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/locations/partners</t>
+  </si>
+  <si>
     <t>addc/en-us/business/help-and-support/account-management-and-bills.report.json</t>
   </si>
   <si>
@@ -295,13 +325,7 @@
     <t>addc/en-us/business/locations/branches.report.json</t>
   </si>
   <si>
-    <t>["hero-text","cards-support"]</t>
-  </si>
-  <si>
     <t>addc/en-us/business/locations/branches</t>
-  </si>
-  <si>
-    <t>locations</t>
   </si>
   <si>
     <t>2026-09-22T06:47:20.889Z</t>
@@ -720,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1073,62 +1097,62 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G14" t="s">
         <v>37</v>
       </c>
       <c r="H14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G15" t="s">
         <v>37</v>
       </c>
       <c r="H15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B16" t="s">
         <v>48</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1137,24 +1161,24 @@
         <v>50</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
         <v>37</v>
       </c>
       <c r="H16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
         <v>48</v>
       </c>
       <c r="C17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1163,24 +1187,24 @@
         <v>50</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
         <v>37</v>
       </c>
       <c r="H17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
         <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -1189,24 +1213,24 @@
         <v>50</v>
       </c>
       <c r="F18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
         <v>37</v>
       </c>
       <c r="H18" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
         <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -1215,30 +1239,30 @@
         <v>50</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G19" t="s">
         <v>37</v>
       </c>
       <c r="H19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="F20" t="s">
         <v>97</v>
@@ -1255,7 +1279,7 @@
         <v>99</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
         <v>100</v>
@@ -1264,7 +1288,7 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="F21" t="s">
         <v>101</v>
@@ -1281,7 +1305,7 @@
         <v>103</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
         <v>104</v>
@@ -1290,7 +1314,7 @@
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="F22" t="s">
         <v>105</v>
@@ -1300,6 +1324,58 @@
       </c>
       <c r="H22" t="s">
         <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H23" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" t="s">
+        <v>112</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" t="s">
+        <v>113</v>
+      </c>
+      <c r="G24" t="s">
+        <v>37</v>
+      </c>
+      <c r="H24" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>